<commit_message>
feat(assets): add download template for data import
</commit_message>
<xml_diff>
--- a/public/template/guest-example.xlsx
+++ b/public/template/guest-example.xlsx
@@ -26,19 +26,60 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ikmal</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>ikmal:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+untuk nomor_undangan tidak wajib diisi (boleh di kosongi)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>nama_utama</t>
   </si>
   <si>
-    <t>Budi Santoso</t>
+    <t>nomor_undangan</t>
   </si>
   <si>
-    <t>Siti Rahayu</t>
+    <t>jumlah_tamu</t>
   </si>
   <si>
-    <t>Ahmad Fauzi</t>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Sparrow</t>
+  </si>
+  <si>
+    <t>NUD-0921</t>
+  </si>
+  <si>
+    <t>Black Devil</t>
   </si>
 </sst>
 </file>
@@ -51,7 +92,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,13 +244,30 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -530,7 +588,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -554,16 +612,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -572,90 +630,93 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1191,31 +1252,52 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="3"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="3" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="20.4375" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.7578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>